<commit_message>
Commit vignette 2's last 29 regenerated files and test every bundle against its metadata
c6f90750 took only 192 of the regeneration pass's 221 changed files: the copy back from
D:\tmp\r62\ocp7 was cut short when its printed output was piped into a reader that closed
early, so vignettes/vignette-2/old_to_new_change_decomposition.csv to
worked_example_size_mismatch.xlsx kept the earlier sample's figures while the bundle's
metadata.json recorded the new fit (adjusted VaR99.5 0.3126 against the run's 0.3129). The
recorded pass of c6f90750 (D:\tmp\r62\ocp8) caught it. The 29 files now hold the
regeneration's bytes, checked after the copy for all 220 copied paths.

test_vignette_bundle_consistency.py recomputes each vignette's size-mismatch multiplier from
its own metadata.json and checks the mix-mismatch overlay's gamma against it: both fail on
vignette 2 at c6f90750 and pass here.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vignettes/vignette-2/old_to_new_change_decomposition.xlsx
+++ b/vignettes/vignette-2/old_to_new_change_decomposition.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.048185</v>
+        <v>0.048499</v>
       </c>
       <c r="C2" t="n">
-        <v>0.050595</v>
+        <v>0.050924</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.00241</v>
+        <v>0.002425</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.237935</v>
+        <v>0.23821</v>
       </c>
       <c r="C3" t="n">
-        <v>0.249837</v>
+        <v>0.250119</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0.011902</v>
+        <v>0.01191</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.297704</v>
+        <v>0.297977</v>
       </c>
       <c r="C4" t="n">
-        <v>0.312595</v>
+        <v>0.312875</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.014891</v>
+        <v>0.014898</v>
       </c>
     </row>
   </sheetData>

</xml_diff>